<commit_message>
Update and restructure analysis and templates
</commit_message>
<xml_diff>
--- a/standalone/analysis/data/mfa.xlsx
+++ b/standalone/analysis/data/mfa.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10830"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11214"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/agamemnon/GitHub/quantrr/standalone/analysis/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F8394077-847C-F540-92FF-B655FCD19518}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DADEB269-8333-C44C-A83F-B535B2096C74}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="60" yWindow="760" windowWidth="28040" windowHeight="17800" activeTab="2" xr2:uid="{48D4EEF9-DFA2-7C44-84E9-995A687A38D6}"/>
+    <workbookView xWindow="60" yWindow="760" windowWidth="28040" windowHeight="17780" activeTab="2" xr2:uid="{48D4EEF9-DFA2-7C44-84E9-995A687A38D6}"/>
   </bookViews>
   <sheets>
     <sheet name="Risks" sheetId="2" r:id="rId1"/>
@@ -43,55 +43,55 @@
     <t>Expert</t>
   </si>
   <si>
+    <t>High (95%)</t>
+  </si>
+  <si>
+    <t>Most Likely</t>
+  </si>
+  <si>
+    <t>Frequency (per yer)</t>
+  </si>
+  <si>
+    <t>Risk</t>
+  </si>
+  <si>
+    <t>Description</t>
+  </si>
+  <si>
+    <t>Cybersecurity Breach</t>
+  </si>
+  <si>
+    <t>Treatment</t>
+  </si>
+  <si>
+    <t>None</t>
+  </si>
+  <si>
+    <t>Current system as it is today</t>
+  </si>
+  <si>
+    <t>IRIS</t>
+  </si>
+  <si>
+    <t>Paper</t>
+  </si>
+  <si>
+    <t>Fully implement MFA for all accounts</t>
+  </si>
+  <si>
+    <t>Risk of a cybersecurity breach</t>
+  </si>
+  <si>
+    <t>Use MFA</t>
+  </si>
+  <si>
+    <t>Use MFA (pessimistic)</t>
+  </si>
+  <si>
+    <t>Use MFA (optomistic)</t>
+  </si>
+  <si>
     <t>Low (5%)</t>
-  </si>
-  <si>
-    <t>High (95%)</t>
-  </si>
-  <si>
-    <t>Most Likely</t>
-  </si>
-  <si>
-    <t>Frequency (per yer)</t>
-  </si>
-  <si>
-    <t>Risk</t>
-  </si>
-  <si>
-    <t>Description</t>
-  </si>
-  <si>
-    <t>Cybersecurity Breach</t>
-  </si>
-  <si>
-    <t>Treatment</t>
-  </si>
-  <si>
-    <t>None</t>
-  </si>
-  <si>
-    <t>Current system as it is today</t>
-  </si>
-  <si>
-    <t>IRIS</t>
-  </si>
-  <si>
-    <t>Paper</t>
-  </si>
-  <si>
-    <t>Fully implement MFA for all accounts</t>
-  </si>
-  <si>
-    <t>Risk of a cybersecurity breach</t>
-  </si>
-  <si>
-    <t>Use MFA</t>
-  </si>
-  <si>
-    <t>Use MFA (pessimistic)</t>
-  </si>
-  <si>
-    <t>Use MFA (optomistic)</t>
   </si>
 </sst>
 </file>
@@ -513,18 +513,18 @@
   <sheetData>
     <row r="1" spans="1:2" s="1" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>5</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>6</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B2" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
   </sheetData>
@@ -543,26 +543,26 @@
   <sheetData>
     <row r="1" spans="1:2" s="1" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
+        <v>8</v>
+      </c>
+      <c r="B2" t="s">
         <v>9</v>
-      </c>
-      <c r="B2" t="s">
-        <v>10</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B3" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
   </sheetData>
@@ -582,96 +582,96 @@
   <sheetData>
     <row r="1" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="D1" s="4" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E1" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="F1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="F1" s="2" t="s">
-        <v>2</v>
-      </c>
       <c r="G1" s="2" t="s">
-        <v>3</v>
+        <v>17</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B2" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C2" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D2" s="5">
         <v>7.4800000000000005E-2</v>
       </c>
       <c r="E2" s="3">
-        <v>31900</v>
+        <v>736000</v>
       </c>
       <c r="F2" s="3">
         <v>17000000</v>
       </c>
       <c r="G2" s="3">
-        <v>736000</v>
+        <v>31900</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B3" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C3" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D3" s="6">
         <f>D$2*(1-0.99)</f>
         <v>7.4800000000000073E-4</v>
       </c>
       <c r="E3" s="3">
-        <v>31900</v>
+        <v>736000</v>
       </c>
       <c r="F3" s="3">
         <v>17000000</v>
       </c>
       <c r="G3" s="3">
-        <v>736000</v>
+        <v>31900</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B4" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C4" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D4" s="6">
         <f>D$2*(1-0.76)</f>
         <v>1.7951999999999999E-2</v>
       </c>
       <c r="E4" s="3">
-        <v>31900</v>
+        <v>736000</v>
       </c>
       <c r="F4" s="3">
         <v>17000000</v>
       </c>
       <c r="G4" s="3">
-        <v>736000</v>
+        <v>31900</v>
       </c>
     </row>
   </sheetData>

</xml_diff>